<commit_message>
Excel's viewer: comments (Excel's notes, threaded comments with their replies, LibreOffice's annotations) — Excel's red corner on the cell, the comment under the cell's words in the bar; links (a cell's hyperlink, a HYPERLINK formula, LibreOffice's) open in their app or go to the sheet and cell they name; ⋯ › Open in another app, Share, About this file, Send log; LibreOffice's number-style colours (a negative's red); a new sheet is never drawn in the last one's order. SheetsTest; checked on the phone (Teo: Check this; To the total → Numbers!B5)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/app/src/test/resources/sheet.xlsx
+++ b/app/src/test/resources/sheet.xlsx
@@ -21,8 +21,51 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:v2="http://schemas.openxmlformats.org/spreadsheetml/2006/main/v2" mc:Ignorable="v2">
+  <authors>
+    <author>Teo</author>
+  </authors>
+  <commentList>
+    <comment ref="A2" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">Check this</t>
+        </r>
+      </text>
+      <mc:AlternateContent>
+        <mc:Choice Requires="v2">
+          <commentPr autoFill="true" autoScale="false" colHidden="false" locked="false" rowHidden="false" textHAlign="justify" textVAlign="top">
+            <anchor moveWithCells="false" sizeWithCells="false">
+              <xdr:from>
+                <xdr:col>1</xdr:col>
+                <xdr:colOff>23</xdr:colOff>
+                <xdr:row>0</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </xdr:from>
+              <xdr:to>
+                <xdr:col>2</xdr:col>
+                <xdr:colOff>47</xdr:colOff>
+                <xdr:row>1</xdr:row>
+                <xdr:rowOff>-15</xdr:rowOff>
+              </xdr:to>
+            </anchor>
+          </commentPr>
+        </mc:Choice>
+        <mc:Fallback/>
+      </mc:AlternateContent>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t xml:space="preserve">Name</t>
   </si>
@@ -49,6 +92,12 @@
   </si>
   <si>
     <t xml:space="preserve">Hello</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To the total</t>
   </si>
   <si>
     <t xml:space="preserve">secret</t>
@@ -64,7 +113,7 @@
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -95,6 +144,12 @@
     <font>
       <i val="true"/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF0000FF"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -154,7 +209,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -177,6 +232,10 @@
     </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -436,6 +495,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Κανονικά"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Κανονικά"&amp;12Σελίδα &amp;P</oddFooter>
   </headerFooter>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -444,7 +504,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="C1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -454,7 +514,19 @@
         <v>8</v>
       </c>
     </row>
+    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A4" r:id="rId1" display="Example"/>
+    <hyperlink ref="B4" location="Numbers!B5" display="To the total"/>
+  </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -475,7 +547,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>